<commit_message>
Re-doing how the data exploration loop works
</commit_message>
<xml_diff>
--- a/assets/per-diem.xlsx
+++ b/assets/per-diem.xlsx
@@ -955,11 +955,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E61"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F61"/>
+  <sheetFormatPr defaultRowHeight="14.5" ns3:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ns3:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -975,8 +975,13 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ExpenseCategory</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ns3:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -992,8 +997,13 @@
       <c r="E2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ns3:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1009,8 +1019,13 @@
       <c r="E3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ns3:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1026,8 +1041,13 @@
       <c r="E4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ns3:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1043,8 +1063,13 @@
       <c r="E5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ns3:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1060,8 +1085,13 @@
       <c r="E6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ns3:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1077,8 +1107,13 @@
       <c r="E7" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ns3:dyDescent="0.35">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1094,8 +1129,13 @@
       <c r="E8" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ns3:dyDescent="0.35">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1111,8 +1151,13 @@
       <c r="E9" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ns3:dyDescent="0.35">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -1128,8 +1173,13 @@
       <c r="E10" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ns3:dyDescent="0.35">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -1145,8 +1195,13 @@
       <c r="E11" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ns3:dyDescent="0.35">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -1162,8 +1217,13 @@
       <c r="E12" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ns3:dyDescent="0.35">
       <c r="A13" t="s">
         <v>38</v>
       </c>
@@ -1179,8 +1239,13 @@
       <c r="E13" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ns3:dyDescent="0.35">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1196,8 +1261,13 @@
       <c r="E14" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ns3:dyDescent="0.35">
       <c r="A15" t="s">
         <v>38</v>
       </c>
@@ -1213,8 +1283,13 @@
       <c r="E15" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ns3:dyDescent="0.35">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -1230,8 +1305,13 @@
       <c r="E16" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ns3:dyDescent="0.35">
       <c r="A17" t="s">
         <v>38</v>
       </c>
@@ -1247,8 +1327,13 @@
       <c r="E17" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ns3:dyDescent="0.35">
       <c r="A18" t="s">
         <v>63</v>
       </c>
@@ -1264,8 +1349,13 @@
       <c r="E18" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ns3:dyDescent="0.35">
       <c r="A19" t="s">
         <v>63</v>
       </c>
@@ -1281,8 +1371,13 @@
       <c r="E19" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ns3:dyDescent="0.35">
       <c r="A20" t="s">
         <v>63</v>
       </c>
@@ -1298,8 +1393,13 @@
       <c r="E20" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ns3:dyDescent="0.35">
       <c r="A21" t="s">
         <v>63</v>
       </c>
@@ -1315,8 +1415,13 @@
       <c r="E21" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ns3:dyDescent="0.35">
       <c r="A22" t="s">
         <v>63</v>
       </c>
@@ -1332,8 +1437,13 @@
       <c r="E22" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ns3:dyDescent="0.35">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -1349,8 +1459,13 @@
       <c r="E23" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ns3:dyDescent="0.35">
       <c r="A24" t="s">
         <v>63</v>
       </c>
@@ -1366,8 +1481,13 @@
       <c r="E24" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ns3:dyDescent="0.35">
       <c r="A25" t="s">
         <v>63</v>
       </c>
@@ -1383,8 +1503,13 @@
       <c r="E25" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ns3:dyDescent="0.35">
       <c r="A26" t="s">
         <v>88</v>
       </c>
@@ -1400,8 +1525,13 @@
       <c r="E26" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ns3:dyDescent="0.35">
       <c r="A27" t="s">
         <v>88</v>
       </c>
@@ -1417,8 +1547,13 @@
       <c r="E27" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ns3:dyDescent="0.35">
       <c r="A28" t="s">
         <v>88</v>
       </c>
@@ -1434,8 +1569,13 @@
       <c r="E28" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ns3:dyDescent="0.35">
       <c r="A29" t="s">
         <v>88</v>
       </c>
@@ -1451,8 +1591,13 @@
       <c r="E29" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ns3:dyDescent="0.35">
       <c r="A30" t="s">
         <v>88</v>
       </c>
@@ -1468,8 +1613,13 @@
       <c r="E30" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ns3:dyDescent="0.35">
       <c r="A31" t="s">
         <v>88</v>
       </c>
@@ -1485,8 +1635,13 @@
       <c r="E31" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ns3:dyDescent="0.35">
       <c r="A32" t="s">
         <v>88</v>
       </c>
@@ -1502,8 +1657,13 @@
       <c r="E32" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ns3:dyDescent="0.35">
       <c r="A33" t="s">
         <v>88</v>
       </c>
@@ -1519,8 +1679,13 @@
       <c r="E33" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ns3:dyDescent="0.35">
       <c r="A34" t="s">
         <v>113</v>
       </c>
@@ -1536,8 +1701,13 @@
       <c r="E34" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ns3:dyDescent="0.35">
       <c r="A35" t="s">
         <v>113</v>
       </c>
@@ -1553,8 +1723,13 @@
       <c r="E35" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ns3:dyDescent="0.35">
       <c r="A36" t="s">
         <v>113</v>
       </c>
@@ -1570,8 +1745,13 @@
       <c r="E36" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ns3:dyDescent="0.35">
       <c r="A37" t="s">
         <v>113</v>
       </c>
@@ -1587,8 +1767,13 @@
       <c r="E37" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ns3:dyDescent="0.35">
       <c r="A38" t="s">
         <v>113</v>
       </c>
@@ -1604,8 +1789,13 @@
       <c r="E38" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ns3:dyDescent="0.35">
       <c r="A39" t="s">
         <v>113</v>
       </c>
@@ -1621,8 +1811,13 @@
       <c r="E39" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ns3:dyDescent="0.35">
       <c r="A40" t="s">
         <v>113</v>
       </c>
@@ -1638,8 +1833,13 @@
       <c r="E40" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ns3:dyDescent="0.35">
       <c r="A41" t="s">
         <v>113</v>
       </c>
@@ -1655,8 +1855,13 @@
       <c r="E41" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ns3:dyDescent="0.35">
       <c r="A42" t="s">
         <v>138</v>
       </c>
@@ -1672,8 +1877,13 @@
       <c r="E42" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ns3:dyDescent="0.35">
       <c r="A43" t="s">
         <v>138</v>
       </c>
@@ -1689,8 +1899,13 @@
       <c r="E43" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ns3:dyDescent="0.35">
       <c r="A44" t="s">
         <v>138</v>
       </c>
@@ -1706,8 +1921,13 @@
       <c r="E44" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ns3:dyDescent="0.35">
       <c r="A45" t="s">
         <v>138</v>
       </c>
@@ -1723,8 +1943,13 @@
       <c r="E45" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ns3:dyDescent="0.35">
       <c r="A46" t="s">
         <v>138</v>
       </c>
@@ -1740,8 +1965,13 @@
       <c r="E46" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ns3:dyDescent="0.35">
       <c r="A47" t="s">
         <v>138</v>
       </c>
@@ -1757,8 +1987,13 @@
       <c r="E47" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ns3:dyDescent="0.35">
       <c r="A48" t="s">
         <v>138</v>
       </c>
@@ -1774,8 +2009,13 @@
       <c r="E48" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ns3:dyDescent="0.35">
       <c r="A49" t="s">
         <v>138</v>
       </c>
@@ -1791,8 +2031,13 @@
       <c r="E49" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ns3:dyDescent="0.35">
       <c r="A50" t="s">
         <v>162</v>
       </c>
@@ -1808,8 +2053,13 @@
       <c r="E50" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ns3:dyDescent="0.35">
       <c r="A51" t="s">
         <v>162</v>
       </c>
@@ -1825,8 +2075,13 @@
       <c r="E51" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ns3:dyDescent="0.35">
       <c r="A52" t="s">
         <v>162</v>
       </c>
@@ -1842,8 +2097,13 @@
       <c r="E52" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ns3:dyDescent="0.35">
       <c r="A53" t="s">
         <v>162</v>
       </c>
@@ -1859,8 +2119,13 @@
       <c r="E53" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ns3:dyDescent="0.35">
       <c r="A54" t="s">
         <v>162</v>
       </c>
@@ -1876,8 +2141,13 @@
       <c r="E54" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ns3:dyDescent="0.35">
       <c r="A55" t="s">
         <v>162</v>
       </c>
@@ -1893,8 +2163,13 @@
       <c r="E55" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Lodging</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ns3:dyDescent="0.35">
       <c r="A56" t="s">
         <v>162</v>
       </c>
@@ -1910,8 +2185,13 @@
       <c r="E56" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ns3:dyDescent="0.35">
       <c r="A57" t="s">
         <v>162</v>
       </c>
@@ -1927,8 +2207,13 @@
       <c r="E57" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ns3:dyDescent="0.35">
       <c r="A58" t="s">
         <v>187</v>
       </c>
@@ -1944,8 +2229,13 @@
       <c r="E58" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ns3:dyDescent="0.35">
       <c r="A59" t="s">
         <v>187</v>
       </c>
@@ -1961,8 +2251,13 @@
       <c r="E59" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ns3:dyDescent="0.35">
       <c r="A60" t="s">
         <v>187</v>
       </c>
@@ -1978,8 +2273,13 @@
       <c r="E60" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ns3:dyDescent="0.35">
       <c r="A61" t="s">
         <v>187</v>
       </c>
@@ -1994,6 +2294,11 @@
       </c>
       <c r="E61" t="s">
         <v>198</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>